<commit_message>
Nuevo formulario de confirmacion de correo
</commit_message>
<xml_diff>
--- a/docs/Cronograma_Actividades_Residencia_GPON_20Sep2026.xlsx
+++ b/docs/Cronograma_Actividades_Residencia_GPON_20Sep2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karen\OneDrive\Documentos\Redes-Mapeo-GPON-FTTx\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65BA391C-FF9D-41DB-A241-AE5FC1CE0B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5A3C4A8-ADBE-4FBD-BDAD-5C4B582A0C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -440,6 +440,13 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -450,39 +457,32 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -797,152 +797,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="15"/>
-      <c r="T1" s="15"/>
-      <c r="U1" s="15"/>
-      <c r="V1" s="15"/>
-      <c r="W1" s="15"/>
-      <c r="X1" s="15"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
     </row>
     <row r="2" spans="1:24" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15"/>
-      <c r="Q2" s="15"/>
-      <c r="R2" s="15"/>
-      <c r="S2" s="15"/>
-      <c r="T2" s="15"/>
-      <c r="U2" s="15"/>
-      <c r="V2" s="15"/>
-      <c r="W2" s="15"/>
-      <c r="X2" s="15"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
-      <c r="S3" s="15"/>
-      <c r="T3" s="15"/>
-      <c r="U3" s="15"/>
-      <c r="V3" s="15"/>
-      <c r="W3" s="15"/>
-      <c r="X3" s="15"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="15"/>
-      <c r="S4" s="15"/>
-      <c r="T4" s="15"/>
-      <c r="U4" s="15"/>
-      <c r="V4" s="15"/>
-      <c r="W4" s="15"/>
-      <c r="X4" s="15"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
     </row>
     <row r="6" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="12" t="s">
+      <c r="B6" s="12"/>
+      <c r="C6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
       <c r="G6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="12" t="s">
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
       <c r="P6" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="12" t="s">
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="12"/>
       <c r="W6" s="1" t="s">
         <v>8</v>
       </c>
@@ -963,7 +963,7 @@
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -1025,7 +1025,7 @@
       </c>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="13" t="s">
         <v>34</v>
       </c>
       <c r="B8" s="4" t="s">
@@ -1054,12 +1054,12 @@
       <c r="W8" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="X8" s="11" t="s">
+      <c r="X8" s="14" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
+      <c r="A9" s="12"/>
       <c r="B9" s="6" t="s">
         <v>38</v>
       </c>
@@ -1083,11 +1083,11 @@
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="12"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="13" t="s">
         <v>39</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1116,12 +1116,12 @@
       <c r="W10" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="X10" s="11" t="s">
+      <c r="X10" s="14" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
+      <c r="A11" s="12"/>
       <c r="B11" s="6" t="s">
         <v>38</v>
       </c>
@@ -1145,11 +1145,11 @@
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
+      <c r="W11" s="12"/>
+      <c r="X11" s="12"/>
     </row>
     <row r="12" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="13" t="s">
         <v>40</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -1178,12 +1178,12 @@
       <c r="W12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="X12" s="11" t="s">
+      <c r="X12" s="14" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
+      <c r="A13" s="12"/>
       <c r="B13" s="6" t="s">
         <v>38</v>
       </c>
@@ -1207,11 +1207,11 @@
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="12"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="13" t="s">
         <v>41</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -1237,15 +1237,15 @@
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
-      <c r="W14" s="18" t="s">
+      <c r="W14" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="X14" s="11" t="s">
+      <c r="X14" s="14" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
+      <c r="A15" s="12"/>
       <c r="B15" s="6" t="s">
         <v>38</v>
       </c>
@@ -1269,11 +1269,11 @@
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="9"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="12"/>
     </row>
     <row r="16" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="13" t="s">
         <v>44</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -1299,15 +1299,15 @@
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
-      <c r="W16" s="8" t="s">
+      <c r="W16" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X16" s="11" t="s">
+      <c r="X16" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
+      <c r="A17" s="12"/>
       <c r="B17" s="6" t="s">
         <v>38</v>
       </c>
@@ -1331,11 +1331,11 @@
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
-      <c r="W17" s="9"/>
-      <c r="X17" s="9"/>
+      <c r="W17" s="12"/>
+      <c r="X17" s="12"/>
     </row>
     <row r="18" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="13" t="s">
         <v>47</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -1361,15 +1361,15 @@
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
-      <c r="W18" s="8" t="s">
+      <c r="W18" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X18" s="11" t="s">
+      <c r="X18" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
+      <c r="A19" s="12"/>
       <c r="B19" s="6" t="s">
         <v>38</v>
       </c>
@@ -1393,11 +1393,11 @@
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
-      <c r="W19" s="9"/>
-      <c r="X19" s="9"/>
+      <c r="W19" s="12"/>
+      <c r="X19" s="12"/>
     </row>
     <row r="20" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="13" t="s">
         <v>48</v>
       </c>
       <c r="B20" s="4" t="s">
@@ -1423,15 +1423,15 @@
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
-      <c r="W20" s="8" t="s">
+      <c r="W20" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X20" s="11" t="s">
+      <c r="X20" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
+      <c r="A21" s="12"/>
       <c r="B21" s="6" t="s">
         <v>38</v>
       </c>
@@ -1455,11 +1455,11 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="9"/>
-      <c r="X21" s="9"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="12"/>
     </row>
     <row r="22" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="13" t="s">
         <v>49</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -1485,15 +1485,15 @@
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
-      <c r="W22" s="8" t="s">
+      <c r="W22" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X22" s="11" t="s">
+      <c r="X22" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
+      <c r="A23" s="12"/>
       <c r="B23" s="6" t="s">
         <v>38</v>
       </c>
@@ -1517,11 +1517,11 @@
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
-      <c r="W23" s="9"/>
-      <c r="X23" s="9"/>
+      <c r="W23" s="12"/>
+      <c r="X23" s="12"/>
     </row>
     <row r="24" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="13" t="s">
         <v>50</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -1547,15 +1547,15 @@
       <c r="T24" s="2"/>
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
-      <c r="W24" s="8" t="s">
+      <c r="W24" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X24" s="11" t="s">
+      <c r="X24" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
+      <c r="A25" s="12"/>
       <c r="B25" s="6" t="s">
         <v>38</v>
       </c>
@@ -1579,11 +1579,11 @@
       <c r="T25" s="2"/>
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
-      <c r="W25" s="9"/>
-      <c r="X25" s="9"/>
+      <c r="W25" s="12"/>
+      <c r="X25" s="12"/>
     </row>
     <row r="26" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="13" t="s">
         <v>51</v>
       </c>
       <c r="B26" s="4" t="s">
@@ -1609,15 +1609,15 @@
       <c r="T26" s="2"/>
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
-      <c r="W26" s="8" t="s">
+      <c r="W26" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X26" s="11" t="s">
+      <c r="X26" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9"/>
+      <c r="A27" s="12"/>
       <c r="B27" s="6" t="s">
         <v>38</v>
       </c>
@@ -1641,11 +1641,11 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
-      <c r="W27" s="9"/>
-      <c r="X27" s="9"/>
+      <c r="W27" s="12"/>
+      <c r="X27" s="12"/>
     </row>
     <row r="28" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
       <c r="B28" s="4" t="s">
@@ -1671,15 +1671,15 @@
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
-      <c r="W28" s="8" t="s">
+      <c r="W28" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X28" s="11" t="s">
+      <c r="X28" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
+      <c r="A29" s="12"/>
       <c r="B29" s="6" t="s">
         <v>38</v>
       </c>
@@ -1703,11 +1703,11 @@
       <c r="T29" s="2"/>
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
-      <c r="W29" s="9"/>
-      <c r="X29" s="9"/>
+      <c r="W29" s="12"/>
+      <c r="X29" s="12"/>
     </row>
     <row r="30" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="13" t="s">
         <v>53</v>
       </c>
       <c r="B30" s="4" t="s">
@@ -1733,15 +1733,15 @@
       <c r="T30" s="2"/>
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
-      <c r="W30" s="8" t="s">
+      <c r="W30" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X30" s="11" t="s">
+      <c r="X30" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
+      <c r="A31" s="12"/>
       <c r="B31" s="6" t="s">
         <v>38</v>
       </c>
@@ -1765,11 +1765,11 @@
       <c r="T31" s="2"/>
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="9"/>
+      <c r="W31" s="12"/>
+      <c r="X31" s="12"/>
     </row>
     <row r="32" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="13" t="s">
         <v>54</v>
       </c>
       <c r="B32" s="4" t="s">
@@ -1795,15 +1795,15 @@
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
-      <c r="W32" s="8" t="s">
+      <c r="W32" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X32" s="11" t="s">
+      <c r="X32" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
+      <c r="A33" s="12"/>
       <c r="B33" s="6" t="s">
         <v>38</v>
       </c>
@@ -1827,11 +1827,11 @@
       <c r="T33" s="2"/>
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
-      <c r="W33" s="9"/>
-      <c r="X33" s="9"/>
+      <c r="W33" s="12"/>
+      <c r="X33" s="12"/>
     </row>
     <row r="34" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+      <c r="A34" s="13" t="s">
         <v>55</v>
       </c>
       <c r="B34" s="4" t="s">
@@ -1857,15 +1857,15 @@
       <c r="T34" s="2"/>
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
-      <c r="W34" s="8" t="s">
+      <c r="W34" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X34" s="11" t="s">
+      <c r="X34" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
+      <c r="A35" s="12"/>
       <c r="B35" s="6" t="s">
         <v>38</v>
       </c>
@@ -1889,11 +1889,11 @@
       <c r="T35" s="2"/>
       <c r="U35" s="2"/>
       <c r="V35" s="2"/>
-      <c r="W35" s="9"/>
-      <c r="X35" s="9"/>
+      <c r="W35" s="12"/>
+      <c r="X35" s="12"/>
     </row>
     <row r="36" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="13" t="s">
         <v>56</v>
       </c>
       <c r="B36" s="4" t="s">
@@ -1919,15 +1919,15 @@
       <c r="T36" s="2"/>
       <c r="U36" s="2"/>
       <c r="V36" s="2"/>
-      <c r="W36" s="8" t="s">
+      <c r="W36" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X36" s="11" t="s">
+      <c r="X36" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="9"/>
+      <c r="A37" s="12"/>
       <c r="B37" s="6" t="s">
         <v>38</v>
       </c>
@@ -1951,11 +1951,11 @@
       <c r="T37" s="2"/>
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
-      <c r="W37" s="9"/>
-      <c r="X37" s="9"/>
+      <c r="W37" s="12"/>
+      <c r="X37" s="12"/>
     </row>
     <row r="38" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="13" t="s">
         <v>57</v>
       </c>
       <c r="B38" s="4" t="s">
@@ -1981,15 +1981,15 @@
       <c r="T38" s="5"/>
       <c r="U38" s="5"/>
       <c r="V38" s="2"/>
-      <c r="W38" s="8" t="s">
+      <c r="W38" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X38" s="11" t="s">
+      <c r="X38" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="9"/>
+      <c r="A39" s="12"/>
       <c r="B39" s="6" t="s">
         <v>38</v>
       </c>
@@ -2013,11 +2013,11 @@
       <c r="T39" s="2"/>
       <c r="U39" s="2"/>
       <c r="V39" s="2"/>
-      <c r="W39" s="9"/>
-      <c r="X39" s="9"/>
+      <c r="W39" s="12"/>
+      <c r="X39" s="12"/>
     </row>
     <row r="40" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
+      <c r="A40" s="13" t="s">
         <v>58</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -2043,15 +2043,15 @@
       <c r="T40" s="2"/>
       <c r="U40" s="2"/>
       <c r="V40" s="5"/>
-      <c r="W40" s="8" t="s">
+      <c r="W40" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="X40" s="11" t="s">
+      <c r="X40" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="41" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="9"/>
+      <c r="A41" s="12"/>
       <c r="B41" s="6" t="s">
         <v>38</v>
       </c>
@@ -2075,46 +2075,69 @@
       <c r="T41" s="2"/>
       <c r="U41" s="2"/>
       <c r="V41" s="2"/>
-      <c r="W41" s="9"/>
-      <c r="X41" s="9"/>
+      <c r="W41" s="12"/>
+      <c r="X41" s="12"/>
     </row>
     <row r="42" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="9"/>
-      <c r="H42" s="9"/>
-      <c r="I42" s="9"/>
-      <c r="J42" s="9"/>
-      <c r="K42" s="9"/>
-      <c r="L42" s="9"/>
-      <c r="M42" s="9"/>
-      <c r="N42" s="9"/>
-      <c r="O42" s="9"/>
-      <c r="P42" s="9"/>
-      <c r="Q42" s="9"/>
-      <c r="R42" s="9"/>
-      <c r="S42" s="9"/>
-      <c r="T42" s="9"/>
-      <c r="U42" s="9"/>
-      <c r="V42" s="9"/>
-      <c r="W42" s="9"/>
-      <c r="X42" s="9"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="12"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="12"/>
+      <c r="M42" s="12"/>
+      <c r="N42" s="12"/>
+      <c r="O42" s="12"/>
+      <c r="P42" s="12"/>
+      <c r="Q42" s="12"/>
+      <c r="R42" s="12"/>
+      <c r="S42" s="12"/>
+      <c r="T42" s="12"/>
+      <c r="U42" s="12"/>
+      <c r="V42" s="12"/>
+      <c r="W42" s="12"/>
+      <c r="X42" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="62">
-    <mergeCell ref="A1:X1"/>
-    <mergeCell ref="W34:W35"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="W28:W29"/>
-    <mergeCell ref="X36:X37"/>
-    <mergeCell ref="W24:W25"/>
-    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="W40:W41"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="W36:W37"/>
+    <mergeCell ref="X16:X17"/>
+    <mergeCell ref="W30:W31"/>
+    <mergeCell ref="X38:X39"/>
+    <mergeCell ref="X40:X41"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="W38:W39"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="X32:X33"/>
+    <mergeCell ref="W20:W21"/>
+    <mergeCell ref="X34:X35"/>
+    <mergeCell ref="W16:W17"/>
+    <mergeCell ref="X24:X25"/>
+    <mergeCell ref="W32:W33"/>
+    <mergeCell ref="X28:X29"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="X22:X23"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="X26:X27"/>
+    <mergeCell ref="W10:W11"/>
+    <mergeCell ref="X12:X13"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="X8:X9"/>
     <mergeCell ref="A42:X42"/>
     <mergeCell ref="W12:W13"/>
     <mergeCell ref="G6:K6"/>
@@ -2131,6 +2154,13 @@
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="W8:W9"/>
     <mergeCell ref="W14:W15"/>
+    <mergeCell ref="A1:X1"/>
+    <mergeCell ref="W34:W35"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="W28:W29"/>
+    <mergeCell ref="X36:X37"/>
+    <mergeCell ref="W24:W25"/>
+    <mergeCell ref="A30:A31"/>
     <mergeCell ref="A3:X3"/>
     <mergeCell ref="W26:W27"/>
     <mergeCell ref="A12:A13"/>
@@ -2140,36 +2170,6 @@
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="A4:X4"/>
     <mergeCell ref="X14:X15"/>
-    <mergeCell ref="X22:X23"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="X26:X27"/>
-    <mergeCell ref="W10:W11"/>
-    <mergeCell ref="X12:X13"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="X32:X33"/>
-    <mergeCell ref="W20:W21"/>
-    <mergeCell ref="X34:X35"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="W16:W17"/>
-    <mergeCell ref="X24:X25"/>
-    <mergeCell ref="W32:W33"/>
-    <mergeCell ref="X28:X29"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="W40:W41"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="W36:W37"/>
-    <mergeCell ref="X16:X17"/>
-    <mergeCell ref="W30:W31"/>
-    <mergeCell ref="X38:X39"/>
-    <mergeCell ref="X40:X41"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="W38:W39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(login): estilizar logo sin caja tosca, quitar Entorno Seguro, corregir doble ojo de contrasenia y anadir exportacion KMZ del mapa
</commit_message>
<xml_diff>
--- a/docs/Cronograma_Actividades_Residencia_GPON_20Sep2026.xlsx
+++ b/docs/Cronograma_Actividades_Residencia_GPON_20Sep2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karen\OneDrive\Documentos\Redes-Mapeo-GPON-FTTx\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5A3C4A8-ADBE-4FBD-BDAD-5C4B582A0C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D6846A-24B2-4DE6-A759-4A8EA8621F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,66 +58,6 @@
     <t>TIPO</t>
   </si>
   <si>
-    <t>SEM 1
-(01-07S)</t>
-  </si>
-  <si>
-    <t>SEM 2
-(08-14S)</t>
-  </si>
-  <si>
-    <t>SEM 3
-(15-21S)</t>
-  </si>
-  <si>
-    <t>SEM 4
-(22-28S)</t>
-  </si>
-  <si>
-    <t>SEM 5
-(29S-05O)</t>
-  </si>
-  <si>
-    <t>SEM 6
-(06-12O)</t>
-  </si>
-  <si>
-    <t>SEM 7
-(13-19O)</t>
-  </si>
-  <si>
-    <t>SEM 8
-(20-26O)</t>
-  </si>
-  <si>
-    <t>SEM 9
-(27O-02N)</t>
-  </si>
-  <si>
-    <t>SEM 10
-(03-09N)</t>
-  </si>
-  <si>
-    <t>SEM 11
-(10-16N)</t>
-  </si>
-  <si>
-    <t>SEM 12
-(17-23N)</t>
-  </si>
-  <si>
-    <t>SEM 13
-(24-30N)</t>
-  </si>
-  <si>
-    <t>SEM 14
-(01-07D)</t>
-  </si>
-  <si>
-    <t>SEM 15
-(08-14D)</t>
-  </si>
-  <si>
     <t>SEM 16
 (15-21D)</t>
   </si>
@@ -226,6 +166,66 @@
   </si>
   <si>
     <t>CRONOGRAMA DE ACTIVIDADES DE RESIDENCIA PROFESIONAL</t>
+  </si>
+  <si>
+    <t>SEM 1
+(01-07)</t>
+  </si>
+  <si>
+    <t>SEM 2
+(08-14)</t>
+  </si>
+  <si>
+    <t>SEM 3
+(15-21)</t>
+  </si>
+  <si>
+    <t>SEM 4
+(22-28)</t>
+  </si>
+  <si>
+    <t>SEM 5
+(29S-05)</t>
+  </si>
+  <si>
+    <t>SEM 6
+(06-12)</t>
+  </si>
+  <si>
+    <t>SEM 7
+(13-19)</t>
+  </si>
+  <si>
+    <t>SEM 8
+(20-26)</t>
+  </si>
+  <si>
+    <t>SEM 9
+(27O-02)</t>
+  </si>
+  <si>
+    <t>SEM 10
+(03-09)</t>
+  </si>
+  <si>
+    <t>SEM 11
+(10-16)</t>
+  </si>
+  <si>
+    <t>SEM 12
+(17-23)</t>
+  </si>
+  <si>
+    <t>SEM 13
+(24-30)</t>
+  </si>
+  <si>
+    <t>SEM 14
+(01-07)</t>
+  </si>
+  <si>
+    <t>SEM 15
+(08-14)</t>
   </si>
 </sst>
 </file>
@@ -330,7 +330,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -375,12 +375,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE600"/>
-        <bgColor rgb="FFFFE600"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFE8F5E9"/>
         <bgColor rgb="FFE8F5E9"/>
       </patternFill>
@@ -389,6 +383,18 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor rgb="FFFFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFFE600"/>
       </patternFill>
     </fill>
   </fills>
@@ -419,7 +425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -437,16 +443,9 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -457,21 +456,28 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -481,7 +487,8 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -797,152 +804,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="19"/>
+      <c r="T1" s="19"/>
+      <c r="U1" s="19"/>
+      <c r="V1" s="19"/>
+      <c r="W1" s="19"/>
+      <c r="X1" s="19"/>
     </row>
     <row r="2" spans="1:24" ht="18" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10"/>
-      <c r="S2" s="10"/>
-      <c r="T2" s="10"/>
-      <c r="U2" s="10"/>
-      <c r="V2" s="10"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
+        <v>46</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
+      <c r="X2" s="19"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10"/>
-      <c r="W3" s="10"/>
-      <c r="X3" s="10"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="10"/>
-      <c r="T4" s="10"/>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="10"/>
-      <c r="X4" s="10"/>
+        <v>44</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
     </row>
     <row r="6" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="9"/>
+      <c r="C6" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="17" t="s">
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="18" t="s">
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="12"/>
-      <c r="P6" s="17" t="s">
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="12"/>
-      <c r="T6" s="18" t="s">
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="U6" s="12"/>
-      <c r="V6" s="12"/>
+      <c r="U6" s="9"/>
+      <c r="V6" s="9"/>
       <c r="W6" s="1" t="s">
         <v>8</v>
       </c>
@@ -958,78 +965,78 @@
         <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="O7" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="R7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="S7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="T7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="U7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="V7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="W7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="X7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="R7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="T7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="U7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="V7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="W7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="X7" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -1051,20 +1058,20 @@
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
-      <c r="W8" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="X8" s="14" t="s">
-        <v>37</v>
+      <c r="W8" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="X8" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
+      <c r="A9" s="9"/>
       <c r="B9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+        <v>23</v>
+      </c>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1083,15 +1090,15 @@
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
-      <c r="W9" s="12"/>
-      <c r="X9" s="12"/>
+      <c r="W9" s="9"/>
+      <c r="X9" s="9"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>39</v>
+      <c r="A10" s="10" t="s">
+        <v>24</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="5"/>
@@ -1113,20 +1120,20 @@
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
-      <c r="W10" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="X10" s="14" t="s">
-        <v>37</v>
+      <c r="W10" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="X10" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
+      <c r="A11" s="9"/>
       <c r="B11" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="7"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1145,15 +1152,15 @@
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
-      <c r="W11" s="12"/>
-      <c r="X11" s="12"/>
+      <c r="W11" s="9"/>
+      <c r="X11" s="9"/>
     </row>
     <row r="12" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
-        <v>40</v>
+      <c r="A12" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -1175,21 +1182,21 @@
       <c r="T12" s="2"/>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
-      <c r="W12" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="X12" s="14" t="s">
-        <v>37</v>
+      <c r="W12" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="X12" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
+      <c r="A13" s="9"/>
       <c r="B13" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="7"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -1207,15 +1214,15 @@
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
-      <c r="W13" s="12"/>
-      <c r="X13" s="12"/>
+      <c r="W13" s="9"/>
+      <c r="X13" s="9"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
-        <v>41</v>
+      <c r="A14" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -1237,21 +1244,21 @@
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
-      <c r="W14" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="X14" s="14" t="s">
-        <v>43</v>
+      <c r="W14" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="X14" s="11" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
+      <c r="A15" s="9"/>
       <c r="B15" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="7"/>
+      <c r="E15" s="24"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -1269,15 +1276,15 @@
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
-      <c r="W15" s="12"/>
-      <c r="X15" s="12"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
     </row>
     <row r="16" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>44</v>
+      <c r="A16" s="10" t="s">
+        <v>29</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -1299,22 +1306,22 @@
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
-      <c r="W16" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X16" s="14" t="s">
-        <v>46</v>
+      <c r="W16" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X16" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
+      <c r="A17" s="9"/>
       <c r="B17" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+      <c r="F17" s="23"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -1331,15 +1338,15 @@
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
-      <c r="W17" s="12"/>
-      <c r="X17" s="12"/>
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
     </row>
     <row r="18" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>47</v>
+      <c r="A18" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -1361,22 +1368,22 @@
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
-      <c r="W18" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X18" s="14" t="s">
-        <v>46</v>
+      <c r="W18" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X18" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
+      <c r="A19" s="9"/>
       <c r="B19" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="F19" s="23"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -1393,15 +1400,15 @@
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
-      <c r="W19" s="12"/>
-      <c r="X19" s="12"/>
+      <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
     </row>
     <row r="20" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
-        <v>48</v>
+      <c r="A20" s="10" t="s">
+        <v>33</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -1423,22 +1430,22 @@
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
-      <c r="W20" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X20" s="14" t="s">
-        <v>46</v>
+      <c r="W20" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X20" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
+      <c r="A21" s="9"/>
       <c r="B21" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+      <c r="F21" s="23"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
@@ -1455,15 +1462,15 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="12"/>
-      <c r="X21" s="12"/>
+      <c r="W21" s="9"/>
+      <c r="X21" s="9"/>
     </row>
     <row r="22" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
-        <v>49</v>
+      <c r="A22" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -1485,23 +1492,23 @@
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
-      <c r="W22" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X22" s="14" t="s">
-        <v>46</v>
+      <c r="W22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X22" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
+      <c r="A23" s="9"/>
       <c r="B23" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+      <c r="G23" s="23"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
@@ -1517,15 +1524,15 @@
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
-      <c r="W23" s="12"/>
-      <c r="X23" s="12"/>
+      <c r="W23" s="9"/>
+      <c r="X23" s="9"/>
     </row>
     <row r="24" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
-        <v>50</v>
+      <c r="A24" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -1547,17 +1554,17 @@
       <c r="T24" s="2"/>
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
-      <c r="W24" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X24" s="14" t="s">
-        <v>46</v>
+      <c r="W24" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X24" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
+      <c r="A25" s="9"/>
       <c r="B25" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1579,15 +1586,15 @@
       <c r="T25" s="2"/>
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
-      <c r="W25" s="12"/>
-      <c r="X25" s="12"/>
+      <c r="W25" s="9"/>
+      <c r="X25" s="9"/>
     </row>
     <row r="26" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>51</v>
+      <c r="A26" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -1609,17 +1616,17 @@
       <c r="T26" s="2"/>
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
-      <c r="W26" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X26" s="14" t="s">
-        <v>46</v>
+      <c r="W26" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X26" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
+      <c r="A27" s="9"/>
       <c r="B27" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -1641,15 +1648,15 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
-      <c r="W27" s="12"/>
-      <c r="X27" s="12"/>
+      <c r="W27" s="9"/>
+      <c r="X27" s="9"/>
     </row>
     <row r="28" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
-        <v>52</v>
+      <c r="A28" s="10" t="s">
+        <v>37</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -1671,17 +1678,17 @@
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
-      <c r="W28" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X28" s="14" t="s">
-        <v>46</v>
+      <c r="W28" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X28" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="12"/>
+      <c r="A29" s="9"/>
       <c r="B29" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1703,15 +1710,15 @@
       <c r="T29" s="2"/>
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
-      <c r="W29" s="12"/>
-      <c r="X29" s="12"/>
+      <c r="W29" s="9"/>
+      <c r="X29" s="9"/>
     </row>
     <row r="30" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>53</v>
+      <c r="A30" s="10" t="s">
+        <v>38</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -1733,17 +1740,17 @@
       <c r="T30" s="2"/>
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
-      <c r="W30" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X30" s="14" t="s">
-        <v>46</v>
+      <c r="W30" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X30" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="12"/>
+      <c r="A31" s="9"/>
       <c r="B31" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -1765,15 +1772,15 @@
       <c r="T31" s="2"/>
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
-      <c r="W31" s="12"/>
-      <c r="X31" s="12"/>
+      <c r="W31" s="9"/>
+      <c r="X31" s="9"/>
     </row>
     <row r="32" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
-        <v>54</v>
+      <c r="A32" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -1795,17 +1802,17 @@
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
-      <c r="W32" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X32" s="14" t="s">
-        <v>46</v>
+      <c r="W32" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X32" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="12"/>
+      <c r="A33" s="9"/>
       <c r="B33" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -1827,15 +1834,15 @@
       <c r="T33" s="2"/>
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
-      <c r="W33" s="12"/>
-      <c r="X33" s="12"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
     </row>
     <row r="34" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
-        <v>55</v>
+      <c r="A34" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -1857,17 +1864,17 @@
       <c r="T34" s="2"/>
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
-      <c r="W34" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X34" s="14" t="s">
-        <v>46</v>
+      <c r="W34" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X34" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12"/>
+      <c r="A35" s="9"/>
       <c r="B35" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1889,15 +1896,15 @@
       <c r="T35" s="2"/>
       <c r="U35" s="2"/>
       <c r="V35" s="2"/>
-      <c r="W35" s="12"/>
-      <c r="X35" s="12"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
     </row>
     <row r="36" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="13" t="s">
-        <v>56</v>
+      <c r="A36" s="10" t="s">
+        <v>41</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -1919,17 +1926,17 @@
       <c r="T36" s="2"/>
       <c r="U36" s="2"/>
       <c r="V36" s="2"/>
-      <c r="W36" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X36" s="14" t="s">
-        <v>46</v>
+      <c r="W36" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X36" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="12"/>
+      <c r="A37" s="9"/>
       <c r="B37" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -1951,15 +1958,15 @@
       <c r="T37" s="2"/>
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
-      <c r="W37" s="12"/>
-      <c r="X37" s="12"/>
+      <c r="W37" s="9"/>
+      <c r="X37" s="9"/>
     </row>
     <row r="38" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="13" t="s">
-        <v>57</v>
+      <c r="A38" s="10" t="s">
+        <v>42</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -1981,17 +1988,17 @@
       <c r="T38" s="5"/>
       <c r="U38" s="5"/>
       <c r="V38" s="2"/>
-      <c r="W38" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X38" s="14" t="s">
-        <v>46</v>
+      <c r="W38" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X38" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="12"/>
+      <c r="A39" s="9"/>
       <c r="B39" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -2013,15 +2020,15 @@
       <c r="T39" s="2"/>
       <c r="U39" s="2"/>
       <c r="V39" s="2"/>
-      <c r="W39" s="12"/>
-      <c r="X39" s="12"/>
+      <c r="W39" s="9"/>
+      <c r="X39" s="9"/>
     </row>
     <row r="40" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="13" t="s">
-        <v>58</v>
+      <c r="A40" s="10" t="s">
+        <v>43</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -2043,17 +2050,17 @@
       <c r="T40" s="2"/>
       <c r="U40" s="2"/>
       <c r="V40" s="5"/>
-      <c r="W40" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="X40" s="14" t="s">
-        <v>46</v>
+      <c r="W40" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="X40" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="12"/>
+      <c r="A41" s="9"/>
       <c r="B41" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -2075,39 +2082,85 @@
       <c r="T41" s="2"/>
       <c r="U41" s="2"/>
       <c r="V41" s="2"/>
-      <c r="W41" s="12"/>
-      <c r="X41" s="12"/>
+      <c r="W41" s="9"/>
+      <c r="X41" s="9"/>
     </row>
     <row r="42" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="12"/>
-      <c r="I42" s="12"/>
-      <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
-      <c r="L42" s="12"/>
-      <c r="M42" s="12"/>
-      <c r="N42" s="12"/>
-      <c r="O42" s="12"/>
-      <c r="P42" s="12"/>
-      <c r="Q42" s="12"/>
-      <c r="R42" s="12"/>
-      <c r="S42" s="12"/>
-      <c r="T42" s="12"/>
-      <c r="U42" s="12"/>
-      <c r="V42" s="12"/>
-      <c r="W42" s="12"/>
-      <c r="X42" s="12"/>
+      <c r="A42" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+      <c r="J42" s="9"/>
+      <c r="K42" s="9"/>
+      <c r="L42" s="9"/>
+      <c r="M42" s="9"/>
+      <c r="N42" s="9"/>
+      <c r="O42" s="9"/>
+      <c r="P42" s="9"/>
+      <c r="Q42" s="9"/>
+      <c r="R42" s="9"/>
+      <c r="S42" s="9"/>
+      <c r="T42" s="9"/>
+      <c r="U42" s="9"/>
+      <c r="V42" s="9"/>
+      <c r="W42" s="9"/>
+      <c r="X42" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="62">
+    <mergeCell ref="A1:X1"/>
+    <mergeCell ref="W34:W35"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="W28:W29"/>
+    <mergeCell ref="X36:X37"/>
+    <mergeCell ref="W24:W25"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A3:X3"/>
+    <mergeCell ref="W26:W27"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A2:X2"/>
+    <mergeCell ref="W22:W23"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="A4:X4"/>
+    <mergeCell ref="X14:X15"/>
+    <mergeCell ref="A42:X42"/>
+    <mergeCell ref="W12:W13"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="X18:X19"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="X20:X21"/>
+    <mergeCell ref="X10:X11"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="X30:X31"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="W18:W19"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="W14:W15"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="X26:X27"/>
+    <mergeCell ref="W10:W11"/>
+    <mergeCell ref="X12:X13"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="W32:W33"/>
+    <mergeCell ref="X28:X29"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="X22:X23"/>
     <mergeCell ref="W40:W41"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="W36:W37"/>
@@ -2124,52 +2177,6 @@
     <mergeCell ref="X34:X35"/>
     <mergeCell ref="W16:W17"/>
     <mergeCell ref="X24:X25"/>
-    <mergeCell ref="W32:W33"/>
-    <mergeCell ref="X28:X29"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="X22:X23"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="X26:X27"/>
-    <mergeCell ref="W10:W11"/>
-    <mergeCell ref="X12:X13"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="A42:X42"/>
-    <mergeCell ref="W12:W13"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="X18:X19"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="X20:X21"/>
-    <mergeCell ref="X10:X11"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="X30:X31"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="W18:W19"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="W8:W9"/>
-    <mergeCell ref="W14:W15"/>
-    <mergeCell ref="A1:X1"/>
-    <mergeCell ref="W34:W35"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="W28:W29"/>
-    <mergeCell ref="X36:X37"/>
-    <mergeCell ref="W24:W25"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A3:X3"/>
-    <mergeCell ref="W26:W27"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A2:X2"/>
-    <mergeCell ref="W22:W23"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="A4:X4"/>
-    <mergeCell ref="X14:X15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Nueva actualizacion de cositas
</commit_message>
<xml_diff>
--- a/docs/Cronograma_Actividades_Residencia_GPON_20Sep2026.xlsx
+++ b/docs/Cronograma_Actividades_Residencia_GPON_20Sep2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karen\OneDrive\Documentos\Redes-Mapeo-GPON-FTTx\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D6846A-24B2-4DE6-A759-4A8EA8621F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2169404-0AFB-4759-93E9-1B5003C69F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -330,7 +330,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -381,12 +381,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor rgb="FFFFF9C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -397,8 +391,20 @@
         <bgColor rgb="FFFFE600"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor rgb="FFFFF9C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -421,11 +427,108 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -443,9 +546,14 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -456,41 +564,72 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -804,152 +943,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
-      <c r="T1" s="19"/>
-      <c r="U1" s="19"/>
-      <c r="V1" s="19"/>
-      <c r="W1" s="19"/>
-      <c r="X1" s="19"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
     </row>
     <row r="2" spans="1:24" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
-    </row>
-    <row r="6" spans="1:24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
+    </row>
+    <row r="6" spans="1:24" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="14" t="s">
+      <c r="B6" s="12"/>
+      <c r="C6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="12" t="s">
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="14" t="s">
+      <c r="H6" s="36"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="12" t="s">
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="14" t="s">
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="12"/>
       <c r="W6" s="1" t="s">
         <v>8</v>
       </c>
@@ -970,19 +1109,19 @@
       <c r="D7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="28" t="s">
         <v>49</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="33" t="s">
         <v>53</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1032,7 +1171,7 @@
       </c>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="4" t="s">
@@ -1042,9 +1181,9 @@
       <c r="D8" s="5"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="34"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -1058,25 +1197,25 @@
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
-      <c r="W8" s="13" t="s">
+      <c r="W8" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="X8" s="11" t="s">
+      <c r="X8" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
+      <c r="A9" s="12"/>
       <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="40"/>
+      <c r="I9" s="34"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -1090,11 +1229,11 @@
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="12"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="13" t="s">
         <v>24</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1102,11 +1241,11 @@
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="40"/>
+      <c r="I10" s="34"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -1120,25 +1259,25 @@
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
-      <c r="W10" s="13" t="s">
+      <c r="W10" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="X10" s="11" t="s">
+      <c r="X10" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
+      <c r="A11" s="12"/>
       <c r="B11" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="34"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -1152,11 +1291,11 @@
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
+      <c r="W11" s="12"/>
+      <c r="X11" s="12"/>
     </row>
     <row r="12" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="13" t="s">
         <v>25</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -1165,10 +1304,10 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="5"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="34"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -1182,25 +1321,25 @@
       <c r="T12" s="2"/>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
-      <c r="W12" s="13" t="s">
+      <c r="W12" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="X12" s="11" t="s">
+      <c r="X12" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
+      <c r="A13" s="12"/>
       <c r="B13" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="34"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1214,11 +1353,11 @@
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="12"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="13" t="s">
         <v>26</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -1228,9 +1367,9 @@
       <c r="D14" s="2"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="34"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -1244,25 +1383,25 @@
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
-      <c r="W14" s="17" t="s">
+      <c r="W14" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="X14" s="11" t="s">
+      <c r="X14" s="14" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
+      <c r="A15" s="12"/>
       <c r="B15" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="34"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -1276,11 +1415,11 @@
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="9"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="12"/>
     </row>
     <row r="16" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="13" t="s">
         <v>29</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -1289,10 +1428,10 @@
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="34"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -1306,25 +1445,25 @@
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
-      <c r="W16" s="8" t="s">
+      <c r="W16" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X16" s="11" t="s">
+      <c r="X16" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
+      <c r="A17" s="12"/>
       <c r="B17" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="34"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
@@ -1338,11 +1477,11 @@
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
-      <c r="W17" s="9"/>
-      <c r="X17" s="9"/>
+      <c r="W17" s="12"/>
+      <c r="X17" s="12"/>
     </row>
     <row r="18" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="13" t="s">
         <v>32</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -1351,10 +1490,10 @@
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="43"/>
+      <c r="I18" s="34"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -1368,25 +1507,25 @@
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
-      <c r="W18" s="8" t="s">
+      <c r="W18" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X18" s="11" t="s">
+      <c r="X18" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
+      <c r="A19" s="12"/>
       <c r="B19" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="34"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -1400,11 +1539,11 @@
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
-      <c r="W19" s="9"/>
-      <c r="X19" s="9"/>
+      <c r="W19" s="12"/>
+      <c r="X19" s="12"/>
     </row>
     <row r="20" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="13" t="s">
         <v>33</v>
       </c>
       <c r="B20" s="4" t="s">
@@ -1414,9 +1553,9 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="2"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="34"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
@@ -1430,25 +1569,25 @@
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
-      <c r="W20" s="8" t="s">
+      <c r="W20" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X20" s="11" t="s">
+      <c r="X20" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
+      <c r="A21" s="12"/>
       <c r="B21" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="34"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -1462,11 +1601,11 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="9"/>
-      <c r="X21" s="9"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="12"/>
     </row>
     <row r="22" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="13" t="s">
         <v>34</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -1476,9 +1615,9 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="5"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="35"/>
       <c r="J22" s="5"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -1492,15 +1631,15 @@
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
-      <c r="W22" s="8" t="s">
+      <c r="W22" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X22" s="11" t="s">
+      <c r="X22" s="14" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
+    <row r="23" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="12"/>
       <c r="B23" s="6" t="s">
         <v>23</v>
       </c>
@@ -1508,9 +1647,9 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="34"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -1524,11 +1663,11 @@
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
-      <c r="W23" s="9"/>
-      <c r="X23" s="9"/>
+      <c r="W23" s="12"/>
+      <c r="X23" s="12"/>
     </row>
     <row r="24" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="13" t="s">
         <v>35</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -1539,7 +1678,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
+      <c r="H24" s="37"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="5"/>
@@ -1554,15 +1693,15 @@
       <c r="T24" s="2"/>
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
-      <c r="W24" s="8" t="s">
+      <c r="W24" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X24" s="11" t="s">
+      <c r="X24" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
+      <c r="A25" s="12"/>
       <c r="B25" s="6" t="s">
         <v>23</v>
       </c>
@@ -1586,11 +1725,11 @@
       <c r="T25" s="2"/>
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
-      <c r="W25" s="9"/>
-      <c r="X25" s="9"/>
+      <c r="W25" s="12"/>
+      <c r="X25" s="12"/>
     </row>
     <row r="26" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="13" t="s">
         <v>36</v>
       </c>
       <c r="B26" s="4" t="s">
@@ -1616,15 +1755,15 @@
       <c r="T26" s="2"/>
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
-      <c r="W26" s="8" t="s">
+      <c r="W26" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X26" s="11" t="s">
+      <c r="X26" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9"/>
+      <c r="A27" s="12"/>
       <c r="B27" s="6" t="s">
         <v>23</v>
       </c>
@@ -1648,11 +1787,11 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
-      <c r="W27" s="9"/>
-      <c r="X27" s="9"/>
+      <c r="W27" s="12"/>
+      <c r="X27" s="12"/>
     </row>
     <row r="28" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="13" t="s">
         <v>37</v>
       </c>
       <c r="B28" s="4" t="s">
@@ -1678,15 +1817,15 @@
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
-      <c r="W28" s="8" t="s">
+      <c r="W28" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X28" s="11" t="s">
+      <c r="X28" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
+      <c r="A29" s="12"/>
       <c r="B29" s="6" t="s">
         <v>23</v>
       </c>
@@ -1710,11 +1849,11 @@
       <c r="T29" s="2"/>
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
-      <c r="W29" s="9"/>
-      <c r="X29" s="9"/>
+      <c r="W29" s="12"/>
+      <c r="X29" s="12"/>
     </row>
     <row r="30" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="13" t="s">
         <v>38</v>
       </c>
       <c r="B30" s="4" t="s">
@@ -1740,15 +1879,15 @@
       <c r="T30" s="2"/>
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
-      <c r="W30" s="8" t="s">
+      <c r="W30" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X30" s="11" t="s">
+      <c r="X30" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
+      <c r="A31" s="12"/>
       <c r="B31" s="6" t="s">
         <v>23</v>
       </c>
@@ -1772,11 +1911,11 @@
       <c r="T31" s="2"/>
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="9"/>
+      <c r="W31" s="12"/>
+      <c r="X31" s="12"/>
     </row>
     <row r="32" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="13" t="s">
         <v>39</v>
       </c>
       <c r="B32" s="4" t="s">
@@ -1802,15 +1941,15 @@
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
-      <c r="W32" s="8" t="s">
+      <c r="W32" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X32" s="11" t="s">
+      <c r="X32" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
+      <c r="A33" s="12"/>
       <c r="B33" s="6" t="s">
         <v>23</v>
       </c>
@@ -1834,11 +1973,11 @@
       <c r="T33" s="2"/>
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
-      <c r="W33" s="9"/>
-      <c r="X33" s="9"/>
+      <c r="W33" s="12"/>
+      <c r="X33" s="12"/>
     </row>
     <row r="34" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+      <c r="A34" s="13" t="s">
         <v>40</v>
       </c>
       <c r="B34" s="4" t="s">
@@ -1864,15 +2003,15 @@
       <c r="T34" s="2"/>
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
-      <c r="W34" s="8" t="s">
+      <c r="W34" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X34" s="11" t="s">
+      <c r="X34" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
+      <c r="A35" s="12"/>
       <c r="B35" s="6" t="s">
         <v>23</v>
       </c>
@@ -1896,11 +2035,11 @@
       <c r="T35" s="2"/>
       <c r="U35" s="2"/>
       <c r="V35" s="2"/>
-      <c r="W35" s="9"/>
-      <c r="X35" s="9"/>
+      <c r="W35" s="12"/>
+      <c r="X35" s="12"/>
     </row>
     <row r="36" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="13" t="s">
         <v>41</v>
       </c>
       <c r="B36" s="4" t="s">
@@ -1926,15 +2065,15 @@
       <c r="T36" s="2"/>
       <c r="U36" s="2"/>
       <c r="V36" s="2"/>
-      <c r="W36" s="8" t="s">
+      <c r="W36" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X36" s="11" t="s">
+      <c r="X36" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="9"/>
+      <c r="A37" s="12"/>
       <c r="B37" s="6" t="s">
         <v>23</v>
       </c>
@@ -1958,11 +2097,11 @@
       <c r="T37" s="2"/>
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
-      <c r="W37" s="9"/>
-      <c r="X37" s="9"/>
+      <c r="W37" s="12"/>
+      <c r="X37" s="12"/>
     </row>
     <row r="38" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="13" t="s">
         <v>42</v>
       </c>
       <c r="B38" s="4" t="s">
@@ -1988,15 +2127,15 @@
       <c r="T38" s="5"/>
       <c r="U38" s="5"/>
       <c r="V38" s="2"/>
-      <c r="W38" s="8" t="s">
+      <c r="W38" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X38" s="11" t="s">
+      <c r="X38" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="9"/>
+      <c r="A39" s="12"/>
       <c r="B39" s="6" t="s">
         <v>23</v>
       </c>
@@ -2020,11 +2159,11 @@
       <c r="T39" s="2"/>
       <c r="U39" s="2"/>
       <c r="V39" s="2"/>
-      <c r="W39" s="9"/>
-      <c r="X39" s="9"/>
+      <c r="W39" s="12"/>
+      <c r="X39" s="12"/>
     </row>
     <row r="40" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
+      <c r="A40" s="13" t="s">
         <v>43</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -2050,15 +2189,15 @@
       <c r="T40" s="2"/>
       <c r="U40" s="2"/>
       <c r="V40" s="5"/>
-      <c r="W40" s="8" t="s">
+      <c r="W40" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="X40" s="11" t="s">
+      <c r="X40" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="9"/>
+      <c r="A41" s="12"/>
       <c r="B41" s="6" t="s">
         <v>23</v>
       </c>
@@ -2082,39 +2221,85 @@
       <c r="T41" s="2"/>
       <c r="U41" s="2"/>
       <c r="V41" s="2"/>
-      <c r="W41" s="9"/>
-      <c r="X41" s="9"/>
+      <c r="W41" s="12"/>
+      <c r="X41" s="12"/>
     </row>
     <row r="42" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
+      <c r="A42" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="9"/>
-      <c r="H42" s="9"/>
-      <c r="I42" s="9"/>
-      <c r="J42" s="9"/>
-      <c r="K42" s="9"/>
-      <c r="L42" s="9"/>
-      <c r="M42" s="9"/>
-      <c r="N42" s="9"/>
-      <c r="O42" s="9"/>
-      <c r="P42" s="9"/>
-      <c r="Q42" s="9"/>
-      <c r="R42" s="9"/>
-      <c r="S42" s="9"/>
-      <c r="T42" s="9"/>
-      <c r="U42" s="9"/>
-      <c r="V42" s="9"/>
-      <c r="W42" s="9"/>
-      <c r="X42" s="9"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="12"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="12"/>
+      <c r="M42" s="12"/>
+      <c r="N42" s="12"/>
+      <c r="O42" s="12"/>
+      <c r="P42" s="12"/>
+      <c r="Q42" s="12"/>
+      <c r="R42" s="12"/>
+      <c r="S42" s="12"/>
+      <c r="T42" s="12"/>
+      <c r="U42" s="12"/>
+      <c r="V42" s="12"/>
+      <c r="W42" s="12"/>
+      <c r="X42" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="62">
+    <mergeCell ref="W40:W41"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="W36:W37"/>
+    <mergeCell ref="X16:X17"/>
+    <mergeCell ref="W30:W31"/>
+    <mergeCell ref="X38:X39"/>
+    <mergeCell ref="X40:X41"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="W38:W39"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="X32:X33"/>
+    <mergeCell ref="W20:W21"/>
+    <mergeCell ref="X34:X35"/>
+    <mergeCell ref="W16:W17"/>
+    <mergeCell ref="X24:X25"/>
+    <mergeCell ref="W32:W33"/>
+    <mergeCell ref="X28:X29"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="X22:X23"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="X26:X27"/>
+    <mergeCell ref="W10:W11"/>
+    <mergeCell ref="X12:X13"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="A42:X42"/>
+    <mergeCell ref="W12:W13"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="X18:X19"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="X20:X21"/>
+    <mergeCell ref="X10:X11"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="X30:X31"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="W18:W19"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="W14:W15"/>
     <mergeCell ref="A1:X1"/>
     <mergeCell ref="W34:W35"/>
     <mergeCell ref="A40:A41"/>
@@ -2131,52 +2316,6 @@
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="A4:X4"/>
     <mergeCell ref="X14:X15"/>
-    <mergeCell ref="A42:X42"/>
-    <mergeCell ref="W12:W13"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="X18:X19"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="X20:X21"/>
-    <mergeCell ref="X10:X11"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="X30:X31"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="W18:W19"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="W8:W9"/>
-    <mergeCell ref="W14:W15"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="X26:X27"/>
-    <mergeCell ref="W10:W11"/>
-    <mergeCell ref="X12:X13"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="W32:W33"/>
-    <mergeCell ref="X28:X29"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="X22:X23"/>
-    <mergeCell ref="W40:W41"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="W36:W37"/>
-    <mergeCell ref="X16:X17"/>
-    <mergeCell ref="W30:W31"/>
-    <mergeCell ref="X38:X39"/>
-    <mergeCell ref="X40:X41"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="W38:W39"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="X32:X33"/>
-    <mergeCell ref="W20:W21"/>
-    <mergeCell ref="X34:X35"/>
-    <mergeCell ref="W16:W17"/>
-    <mergeCell ref="X24:X25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>